<commit_message>
paper run 2026-09-17 11:55
</commit_message>
<xml_diff>
--- a/reports/2026-09-17.xlsx
+++ b/reports/2026-09-17.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -632,13 +632,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>36.38</v>
+        <v>79.81999999999999</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -658,13 +658,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>36.38</v>
+        <v>79.81999999999999</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -680,7 +680,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -690,7 +690,7 @@
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>36.38</v>
+        <v>43.44</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -699,163 +699,182 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>36.38</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>NO_LIQUIDITY</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" t="n">
-        <v>36.38</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="B22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>79.81999999999999</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>По активам</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>По окнам</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>По часам</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>По цене входа</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>По силе движения</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>

</xml_diff>

<commit_message>
paper run 2026-09-17 17:55
</commit_message>
<xml_diff>
--- a/reports/2026-09-17.xlsx
+++ b/reports/2026-09-17.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,92 @@
         <is>
           <t>P&amp;L $</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-17T15:08:56.416337+00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F2" t="n">
+        <v>22.35</v>
+      </c>
+      <c r="G2" t="n">
+        <v>43.83</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>21.48</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-17T17:12:44.319834+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F3" t="n">
+        <v>38.25</v>
+      </c>
+      <c r="G3" t="n">
+        <v>65.95</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.792</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.00123</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>27.7</v>
       </c>
     </row>
   </sheetData>
@@ -485,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,7 +593,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -517,7 +603,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -536,6 +622,9 @@
           <t>winrate</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -544,7 +633,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>49.18</v>
       </c>
     </row>
     <row r="7">
@@ -554,7 +643,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>49.18</v>
       </c>
     </row>
     <row r="8">
@@ -573,6 +662,9 @@
           <t>pf</t>
         </is>
       </c>
+      <c r="B9" t="n">
+        <v>99</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -581,7 +673,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1061.83</v>
+        <v>1111.01</v>
       </c>
     </row>
     <row r="12">
@@ -632,161 +724,196 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>79.81999999999999</v>
+        <v>153.4</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>27.7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>51.01</v>
+      </c>
+      <c r="E16" t="n">
+        <v>21.48</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>2</v>
-      </c>
-      <c r="C17" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" t="n">
-        <v>79.81999999999999</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
+          <t>По активам</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>39.22</v>
+      </c>
+      <c r="E18" t="n">
+        <v>27.7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>43.44</v>
+        <v>165.19</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>21.48</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" t="n">
-        <v>36.38</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>94.45</v>
+      </c>
+      <c r="E21" t="n">
+        <v>21.48</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>79.81999999999999</v>
+        <v>109.96</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>27.7</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" t="n">
+        <v>114.18</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" t="n">
+        <v>90.23</v>
+      </c>
+      <c r="E25" t="n">
+        <v>49.18</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>REALIZED (реальные сделки)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>По активам</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
@@ -795,42 +922,52 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>27.7</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>21.48</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
@@ -839,45 +976,249 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>27.7</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>21.48</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>21.48</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>27.7</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>21.48</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>27.7</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>По силе движения</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>21.48</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>27.7</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>27.7</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>21.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-17 23:54
</commit_message>
<xml_diff>
--- a/reports/2026-09-17.xlsx
+++ b/reports/2026-09-17.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,92 @@
       </c>
       <c r="K3" t="n">
         <v>27.7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-17T19:41:47.714896+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F4" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>48</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.773</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0.00124</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>21.6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-17T22:11:16.483567+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.759</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.00112</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>4.5</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,7 +679,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -603,7 +689,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -633,7 +719,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>49.18</v>
+        <v>75.28</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +729,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>49.18</v>
+        <v>75.28</v>
       </c>
     </row>
     <row r="8">
@@ -673,7 +759,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1111.01</v>
+        <v>1137.11</v>
       </c>
     </row>
     <row r="12">
@@ -724,16 +810,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D15" t="n">
-        <v>153.4</v>
+        <v>289.5</v>
       </c>
       <c r="E15" t="n">
-        <v>27.7</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="16">
@@ -769,16 +855,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>39.22</v>
+        <v>84.67</v>
       </c>
       <c r="E18" t="n">
-        <v>27.7</v>
+        <v>49.3</v>
       </c>
     </row>
     <row r="19">
@@ -788,16 +874,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D19" t="n">
-        <v>165.19</v>
+        <v>255.84</v>
       </c>
       <c r="E19" t="n">
-        <v>21.48</v>
+        <v>25.98</v>
       </c>
     </row>
     <row r="20">
@@ -814,16 +900,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D21" t="n">
-        <v>94.45</v>
+        <v>230.55</v>
       </c>
       <c r="E21" t="n">
-        <v>21.48</v>
+        <v>47.58</v>
       </c>
     </row>
     <row r="22">
@@ -859,13 +945,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D24" t="n">
-        <v>114.18</v>
+        <v>160.69</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -878,16 +964,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D25" t="n">
-        <v>90.23</v>
+        <v>179.82</v>
       </c>
       <c r="E25" t="n">
-        <v>49.18</v>
+        <v>75.28</v>
       </c>
     </row>
     <row r="27">
@@ -926,13 +1012,13 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>27.7</v>
+        <v>49.3</v>
       </c>
     </row>
     <row r="31">
@@ -942,13 +1028,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" t="n">
-        <v>21.48</v>
+        <v>25.98</v>
       </c>
     </row>
     <row r="33">
@@ -980,13 +1066,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D34" t="n">
-        <v>27.7</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="35">
@@ -1059,166 +1145,198 @@
         <v>27.7</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>21.6</v>
+      </c>
+    </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" t="n">
-        <v>21.48</v>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>4.5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" t="n">
-        <v>27.7</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C44" t="n">
+        <v>3</v>
+      </c>
+      <c r="D44" t="n">
+        <v>47.58</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" t="n">
-        <v>21.48</v>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>27.7</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>1</v>
-      </c>
-      <c r="C47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" t="n">
-        <v>27.7</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" t="n">
+        <v>25.98</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>1</v>
-      </c>
-      <c r="C50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" t="n">
-        <v>27.7</v>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="n">
+        <v>2</v>
+      </c>
+      <c r="D49" t="n">
+        <v>49.3</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2</v>
+      </c>
+      <c r="C52" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" t="n">
+        <v>49.3</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B51" t="n">
-        <v>1</v>
-      </c>
-      <c r="C51" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" t="n">
-        <v>21.48</v>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" t="n">
+        <v>25.98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>